<commit_message>
fix(pinout): pin name first in GPIO names, then mux functions
</commit_message>
<xml_diff>
--- a/pinout/fc7300-320-pin-a1.xlsx
+++ b/pinout/fc7300-320-pin-a1.xlsx
@@ -421,7 +421,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>DISABLED/PTA0/FTU4_CH6/FLEXCAN5_RX/SENT1_RXD2/FTU2_QD_PHA/FCUART0_CTS/TRGSEL_OUT3</t>
+          <t>PTA0/DISABLED/FTU4_CH6/FLEXCAN5_RX/SENT1_RXD2/FTU2_QD_PHA/FCUART0_CTS/TRGSEL_OUT3</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DISABLED/PTA1/FTU4_CH4/FCUART15_RX/SENT1_RXD0/FTU1_QD_PHA/FCUART0_RTS/TRGSEL_OUT0</t>
+          <t>PTA1/DISABLED/FTU4_CH4/FCUART15_RX/SENT1_RXD0/FTU1_QD_PHA/FCUART0_RTS/TRGSEL_OUT0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -475,7 +475,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DISABLED/PTA2/FTU2_CH3/FCIIC0_SDA/MSC1_FCLP/FCUART0_RX</t>
+          <t>PTA2/DISABLED/FTU2_CH3/FCIIC0_SDA/MSC1_FCLP/FCUART0_RX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DISABLED/PTA3/FTU2_CH2/FCIIC0_SCL/FCUART0_TX</t>
+          <t>PTA3/DISABLED/FTU2_CH2/FCIIC0_SCL/FCUART0_TX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JTAG_TMS/SWD_DIO/PTA4/CMP0_OUT</t>
+          <t>PTA4/JTAG_TMS/SWD_DIO/CMP0_OUT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -556,7 +556,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADC2_SE13/PTA6/FTU5_CH0/FTU_FLT13/FCUART1_CTS/TRGSEL_OUT4/SDDF0_CH0/FCSPI7_SIN</t>
+          <t>PTA6/ADC2_SE13/FTU5_CH0/FTU_FLT13/FCUART1_CTS/TRGSEL_OUT4/SDDF0_CH0/FCSPI7_SIN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -583,7 +583,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADC2_SE11/PTA7/FTU7_CH6/FTU_FLT12/FCUART1_RTS/FCSPI4_SIN</t>
+          <t>PTA7/ADC2_SE11/FTU7_CH6/FTU_FLT12/FCUART1_RTS/FCSPI4_SIN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -610,7 +610,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADC1_SE14/PTA8/FCUART2_RX</t>
+          <t>PTA8/ADC1_SE14/FCUART2_RX</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -637,7 +637,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADC1_SE15/PTA9/FCUART2_TX/RTC_CLKOUT</t>
+          <t>PTA9/ADC1_SE15/FCUART2_TX/RTC_CLKOUT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -664,7 +664,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JTAG_TDO/PTA10/FTU3_CH1</t>
+          <t>PTA10/JTAG_TDO/FTU3_CH1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DISABLED/PTA11/FTU3_CH0/FLEXCAN1_TX/FCSPI0_PCS3/NMI_b</t>
+          <t>PTA11/DISABLED/FTU3_CH0/FLEXCAN1_TX/FCSPI0_PCS3/NMI_b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -718,7 +718,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADC1_SE18/PTA12/FTU0_CH7/FLEXCAN1_RX/CMP2_OUT/FCSPI0_SOUT/FTU2_QD_PHB</t>
+          <t>PTA12/ADC1_SE18/FTU0_CH7/FLEXCAN1_RX/CMP2_OUT/FCSPI0_SOUT/FTU2_QD_PHB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -745,7 +745,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DISABLED/PTA13/FTU0_CH3/CMP1_OUT/FCUART0_RX/FTU2_QD_PHA</t>
+          <t>PTA13/DISABLED/FTU0_CH3/CMP1_OUT/FCUART0_RX/FTU2_QD_PHA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -772,7 +772,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DISABLED/PTA14/FTU_FLT17/AONTIMER0_CLK1/CMP1_OUT/FCUART0_TX</t>
+          <t>PTA14/DISABLED/FTU_FLT17/AONTIMER0_CLK1/CMP1_OUT/FCUART0_TX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -799,7 +799,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADC1_SE28/PTA15/FTU6_CH4/FTU5_QD_PHB/FCUART10_TX/TRGSEL_OUT0/FLEXCAN3_RX</t>
+          <t>PTA15/ADC1_SE28/FTU6_CH4/FTU5_QD_PHB/FCUART10_TX/TRGSEL_OUT0/FLEXCAN3_RX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DISABLED/PTA16/FTU6_CH2/FCSMU_PIN0</t>
+          <t>PTA16/DISABLED/FTU6_CH2/FCSMU_PIN0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -853,7 +853,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADC2_SE19/PTA17/FTU5_CH5/FTU_FLT15/FCSPI1_PCS2/FLEXCAN4_TX</t>
+          <t>PTA17/ADC2_SE19/FTU5_CH5/FTU_FLT15/FCSPI1_PCS2/FLEXCAN4_TX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADC1_SE7/PTA18/FTU3_CH6/FCUART1_TX</t>
+          <t>PTA18/ADC1_SE7/FTU3_CH6/FCUART1_TX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ADC1_SE3/PTA19/FCUART1_RX/FTU6_CH7</t>
+          <t>PTA19/ADC1_SE3/FCUART1_RX/FTU6_CH7</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -934,7 +934,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ADC1_SE6/PTA20/FTU3_CH7/FCUART3_RTS</t>
+          <t>PTA20/ADC1_SE6/FTU3_CH7/FCUART3_RTS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ADC0_SE2/PTA21/FCUART6_RX/FCUART3_CTS/FTU2_CH5</t>
+          <t>PTA21/ADC0_SE2/FCUART6_RX/FCUART3_CTS/FTU2_CH5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -988,7 +988,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ADC0_SE1/PTA22/FTU2_CH3/FTU2_QD_PHA/FCUART7_RX</t>
+          <t>PTA22/ADC0_SE1/FTU2_CH3/FTU2_QD_PHA/FCUART7_RX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1015,7 +1015,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ADC0_SE14/CMP0_IN6/PTA23/FTU4_CH1/FCUART3_RX/TRACE_D0/FTU4_QD_PHA</t>
+          <t>PTA23/ADC0_SE14/CMP0_IN6/FTU4_CH1/FCUART3_RX/TRACE_D0/FTU4_QD_PHA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ADC0_SE15/CMP0_IN7/PTA24/FTU4_CH0/FCUART3_TX/TRACE_D1/FTU4_QD_PHB</t>
+          <t>PTA24/ADC0_SE15/CMP0_IN7/FTU4_CH0/FCUART3_TX/TRACE_D1/FTU4_QD_PHB</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADC0_SE11/PTA25/FTU4_CH3/FCSPI2_SOUT</t>
+          <t>PTA25/ADC0_SE11/FTU4_CH3/FCSPI2_SOUT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1096,7 +1096,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CMP0_IN1/PTA26/FTU2_CH2</t>
+          <t>PTA26/CMP0_IN1/FTU2_CH2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1123,7 +1123,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ADC0_SE16/PTA27/FTU5_CH7/FCUART0_TX/TRACE_D2/FCSPI1_PCS0</t>
+          <t>PTA27/ADC0_SE16/FTU5_CH7/FCUART0_TX/TRACE_D2/FCSPI1_PCS0</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ADC0_SE18/PTA28/FTU5_CH5/FCUART0_RX/FCSPI1_SCK</t>
+          <t>PTA28/ADC0_SE18/FTU5_CH5/FCUART0_RX/FCSPI1_SCK</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1177,7 +1177,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ADC0_SE19/PTA29/FTU5_CH4/FCSPI1_SIN</t>
+          <t>PTA29/ADC0_SE19/FTU5_CH4/FCSPI1_SIN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1204,7 +1204,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ADC0_SE25/PTA30/FTU5_CH2/FCUART2_RX/TRACE_D5/FCSPI1_PCS2/FTU5_QD_PHB</t>
+          <t>PTA30/ADC0_SE25/FTU5_CH2/FCUART2_RX/TRACE_D5/FCSPI1_PCS2/FTU5_QD_PHB</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1231,7 +1231,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ADC0_SE29/PTA31/FTU0_CH6/FCUART5_TX/FTU_FLT3/FLEXCAN3_TX</t>
+          <t>PTA31/ADC0_SE29/FTU0_CH6/FCUART5_TX/FTU_FLT3/FLEXCAN3_TX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ADC3_SE18/PTB0/SDDF0_BREAK3/FCUART14_TX/FLEXCAN0_RX/FTU3_CH6</t>
+          <t>PTB0/ADC3_SE18/SDDF0_BREAK3/FCUART14_TX/FLEXCAN0_RX/FTU3_CH6</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ADC3_SE17/PTB1/SDDF0_BREAK2/FTU_TCK0/FCUART14_RX/FLEXCAN0_TX/FTU3_CH5</t>
+          <t>PTB1/ADC3_SE17/SDDF0_BREAK2/FTU_TCK0/FCUART14_RX/FLEXCAN0_TX/FTU3_CH5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1312,7 +1312,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ADC3_SE20/PTB3/FTU1_QD_PHA/FCSPI2_SCK/FTU3_CH7</t>
+          <t>PTB3/ADC3_SE20/FTU1_QD_PHA/FCSPI2_SCK/FTU3_CH7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1339,7 +1339,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DISABLED/PTB4/FTU7_CH7/FCUART9_RX/ENET_MDIO</t>
+          <t>PTB4/DISABLED/FTU7_CH7/FCUART9_RX/ENET_MDIO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1366,7 +1366,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DISABLED/PTB5/FTU6_CH2/FCIIC1_SDA/ENET_MDC</t>
+          <t>PTB5/DISABLED/FTU6_CH2/FCIIC1_SDA/ENET_MDC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1393,7 +1393,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>XTAL/PTB6</t>
+          <t>PTB6/XTAL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1420,7 +1420,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>EXTAL/PTB7</t>
+          <t>PTB7/EXTAL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1447,7 +1447,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DISABLED/PTB8/FTU4_CH2/FLEXCAN4_TX/FCUART11_RX/MSC1_SDI0/FCUART1_CTS</t>
+          <t>PTB8/DISABLED/FTU4_CH2/FLEXCAN4_TX/FCUART11_RX/MSC1_SDI0/FCUART1_CTS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1474,7 +1474,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DISABLED/PTB9/FTU2_CH7/FCUART12_TX/TRGSEL_OUT1</t>
+          <t>PTB9/DISABLED/FTU2_CH7/FCUART12_TX/TRGSEL_OUT1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DISABLED/PTB10/FTU2_CH5/TRGSEL_OUT2/FLEXCAN7_RX</t>
+          <t>PTB10/DISABLED/FTU2_CH5/TRGSEL_OUT2/FLEXCAN7_RX</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1528,7 +1528,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ADC2_SE29/PTB12/FTU9_CH3/FLEXCAN2_RX</t>
+          <t>PTB12/ADC2_SE29/FTU9_CH3/FLEXCAN2_RX</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1550,7 +1550,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ADC2_SE28/PTB13/FTU3_CH2/MSC1_SDI3/FCUART16_TX</t>
+          <t>PTB13/ADC2_SE28/FTU3_CH2/MSC1_SDI3/FCUART16_TX</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ADC2_SE27/PTB14/FTU3_CH1/FCUART4_RX/MSC1_EN3</t>
+          <t>PTB14/ADC2_SE27/FTU3_CH1/FCUART4_RX/MSC1_EN3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1604,7 +1604,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ADC2_SE26/PTB15/FTU3_CH0/FCUART4_TX/MSC1_SDI2</t>
+          <t>PTB15/ADC2_SE26/FTU3_CH0/FCUART4_TX/MSC1_SDI2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ADC2_SE25/PTB16/FTU5_CH7/FCUART5_CTS/MSC1_EN2</t>
+          <t>PTB16/ADC2_SE25/FTU5_CH7/FCUART5_CTS/MSC1_EN2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1658,7 +1658,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ADC2_SE20/PTB17/FTU5_CH6/FCSPI1_PCS3/FLEXCAN4_RX/SDDF0_CLK3</t>
+          <t>PTB17/ADC2_SE20/FTU5_CH6/FCSPI1_PCS3/FLEXCAN4_RX/SDDF0_CLK3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1685,7 +1685,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ADC0_SE30/PTB18/FTU0_CH5/FCUART5_RX/FLEXCAN3_RX</t>
+          <t>PTB18/ADC0_SE30/FTU0_CH5/FCUART5_RX/FLEXCAN3_RX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1712,7 +1712,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ADC0_SE31/PTB19/FTU0_CH4</t>
+          <t>PTB19/ADC0_SE31/FTU0_CH4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ADC3_SE31/CMP2_IN0/PTB20/FTU1_CH0/FCUART1_TX/ENET_PPS0/SCG_CLKOUT</t>
+          <t>PTB20/ADC3_SE31/CMP2_IN0/FTU1_CH0/FCUART1_TX/ENET_PPS0/SCG_CLKOUT</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1766,7 +1766,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ADC3_SE30/CMP2_IN1/PTB21/FTU1_CH1/FCUART1_RX/ENET_PPS1/RTC_CLKOUT</t>
+          <t>PTB21/ADC3_SE30/CMP2_IN1/FTU1_CH1/FCUART1_RX/ENET_PPS1/RTC_CLKOUT</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1793,7 +1793,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DISABLED/PTB22/FTU8_CH3/FCUART1_TX/TRACE_D5/OSPI_A_IO0/FCSPI3_PCS2</t>
+          <t>PTB22/DISABLED/FTU8_CH3/FCUART1_TX/TRACE_D5/OSPI_A_IO0/FCSPI3_PCS2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1820,7 +1820,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DISABLED/PTB23/FTU_FLT9/FCSPI2_PCS0/FTU7_CH3/ENET_RXD3</t>
+          <t>PTB23/DISABLED/FTU_FLT9/FCSPI2_PCS0/FTU7_CH3/ENET_RXD3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ADC3_SE29/CMP2_IN2/PTB24/FTU1_CH2</t>
+          <t>PTB24/ADC3_SE29/CMP2_IN2/FTU1_CH2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1874,7 +1874,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ADC3_SE19/PTB25/FCSPI2_PCS0/FTU3_CH6</t>
+          <t>PTB25/ADC3_SE19/FCSPI2_PCS0/FTU3_CH6</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DISABLED/PTB26/FTU6_CH0/ENET_COL/FCSPI3_SIN</t>
+          <t>PTB26/DISABLED/FTU6_CH0/ENET_COL/FCSPI3_SIN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1928,7 +1928,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ADC3_SE21/PTB27/FTU7_CH0/FTU1_QD_PHB/FCSPI2_SOUT</t>
+          <t>PTB27/ADC3_SE21/FTU7_CH0/FTU1_QD_PHB/FCSPI2_SOUT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1955,7 +1955,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ADC3_SE22/PTB28/FTU7_CH1/FCSPI2_SIN</t>
+          <t>PTB28/ADC3_SE22/FTU7_CH1/FCSPI2_SIN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ADC3_SE0/PTB29/FTU1_CH3/FCUART12_RX/MSC0_FCLP</t>
+          <t>PTB29/ADC3_SE0/FTU1_CH3/FCUART12_RX/MSC0_FCLP</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2009,7 +2009,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DISABLED/PTB30/FTU6_CH1/FCIIC1_SCL/FCUART12_TX/ENET_CRS/FCSPI3_SOUT</t>
+          <t>PTB30/DISABLED/FTU6_CH1/FCIIC1_SCL/FCUART12_TX/ENET_CRS/FCSPI3_SOUT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2036,7 +2036,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DISABLED/PTB31/FTU7_CH1/FCSPI2_SCK/ENET_RXD1</t>
+          <t>PTB31/DISABLED/FTU7_CH1/FCSPI2_SCK/ENET_RXD1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2063,7 +2063,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DISABLED/PTC0/FTU8_CH6/TRACE_D6/ENET_RXD1/OSPI_A_IO3/FCSPI3_PCS1</t>
+          <t>PTC0/DISABLED/FTU8_CH6/TRACE_D6/ENET_RXD1/OSPI_A_IO3/FCSPI3_PCS1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2090,7 +2090,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DISABLED/PTC1/FTU7_CH5/ENET_RXD0/OSPI_A_IO2/FCSPI3_PCS0</t>
+          <t>PTC1/DISABLED/FTU7_CH5/ENET_RXD0/OSPI_A_IO2/FCSPI3_PCS0</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DISABLED/PTC2/FTU6_CH3/FCUART0_RX/TRACE_CLKOUT/ENET_TXD0</t>
+          <t>PTC2/DISABLED/FTU6_CH3/FCUART0_RX/TRACE_CLKOUT/ENET_TXD0</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2144,7 +2144,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DISABLED/PTC3/FTU6_CH2/FCUART0_TX/FCSPI3_PCS0</t>
+          <t>PTC3/DISABLED/FTU6_CH2/FCUART0_TX/FCSPI3_PCS0</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2171,7 +2171,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JTAG_TCLK/SWD_CLK/PTC4/FTU3_CH4/FTU1_QD_PHB</t>
+          <t>PTC4/JTAG_TCLK/SWD_CLK/FTU3_CH4/FTU1_QD_PHB</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2198,7 +2198,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>JTAG_TDI/PTC5/FTU3_CH3/FTU1_QD_PHA</t>
+          <t>PTC5/JTAG_TDI/FTU3_CH3/FTU1_QD_PHA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2225,7 +2225,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DISABLED/PTC6/FCUART1_RX/FTU3_CH2/FTU1_QD_PHB</t>
+          <t>PTC6/DISABLED/FCUART1_RX/FTU3_CH2/FTU1_QD_PHB</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ADC1_SE30/PTC7/FCUART1_TX/FTU3_CH3</t>
+          <t>PTC7/ADC1_SE30/FCUART1_TX/FTU3_CH3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ADC2_SE9/PTC8/FTU7_CH4/FTU_FLT11/FTU4_QD_PHB/FCSPI4_PCS0/FCUART0_CTS</t>
+          <t>PTC8/ADC2_SE9/FTU7_CH4/FTU_FLT11/FTU4_QD_PHB/FCSPI4_PCS0/FCUART0_CTS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ADC2_SE8/PTC9/FTU7_CH3/FTU_FLT10/FTU4_QD_PHA/FCSPI4_SCK/FCUART0_RTS</t>
+          <t>PTC9/ADC2_SE8/FTU7_CH3/FTU_FLT10/FTU4_QD_PHA/FCSPI4_SCK/FCUART0_RTS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2333,7 +2333,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ADC2_SE3/PTC10/FTU3_CH4/FLEXCAN4_RX/FCUART13_TX/MSC0_EN1</t>
+          <t>PTC10/ADC2_SE3/FTU3_CH4/FLEXCAN4_RX/FCUART13_TX/MSC0_EN1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2360,7 +2360,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ADC2_SE6/PTC11/FTU3_CH3/FLEXCAN4_TX/FCUART13_RX/MSC0_EN0</t>
+          <t>PTC11/ADC2_SE6/FTU3_CH3/FLEXCAN4_TX/FCUART13_RX/MSC0_EN0</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ADC3_SE1/PTC12/FTU1_CH5/TRGSEL_OUT5/FLEXCAN5_RX/MSC0_EN2</t>
+          <t>PTC12/ADC3_SE1/FTU1_CH5/TRGSEL_OUT5/FLEXCAN5_RX/MSC0_EN2</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2414,7 +2414,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ADC3_SE4/PTC13/FTU1_CH4/TRGSEL_OUT6/FLEXCAN5_TX/MSC0_SOP</t>
+          <t>PTC13/ADC3_SE4/FTU1_CH4/TRGSEL_OUT6/FLEXCAN5_TX/MSC0_SOP</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2441,7 +2441,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DISABLED/PTC14/FTU7_CH4/FCUART1_RX/FCIIC1_SDA/OSPI_A_RWDS</t>
+          <t>PTC14/DISABLED/FTU7_CH4/FCUART1_RX/FCIIC1_SDA/OSPI_A_RWDS</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2468,7 +2468,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DISABLED/PTC15/FTU8_CH4/FCSPI2_PCS3/SCG_CLKOUT/ENET_RXD3/OSPI_A_IO1/FCSPI3_PCS3</t>
+          <t>PTC15/DISABLED/FTU8_CH4/FCSPI2_PCS3/SCG_CLKOUT/ENET_RXD3/OSPI_A_IO1/FCSPI3_PCS3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DISABLED/PTC16/FTU_FLT7/FCSPI2_SOUT/TRGSEL_OUT7/ENET_RXD0/FCUART5_RX</t>
+          <t>PTC16/DISABLED/FTU_FLT7/FCSPI2_SOUT/TRGSEL_OUT7/ENET_RXD0/FCUART5_RX</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2522,7 +2522,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DISABLED/PTC17/FTU_FLT6/TRGSEL_OUT6/ENET_RX_ER/FCUART5_TX</t>
+          <t>PTC17/DISABLED/FTU_FLT6/TRGSEL_OUT6/ENET_RX_ER/FCUART5_TX</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2549,7 +2549,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DISABLED/PTC18/FTU7_CH2/FCSPI2_SIN/ENET_RXD2</t>
+          <t>PTC18/DISABLED/FTU7_CH2/FCSPI2_SIN/ENET_RXD2</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2576,7 +2576,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ADC3_SE5/PTC19/FTU1_CH6/FLEXCAN6_TX/MSC0_EN3</t>
+          <t>PTC19/ADC3_SE5/FTU1_CH6/FLEXCAN6_TX/MSC0_EN3</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ADC3_SE2/PTC20/FTU1_CH7/FLEXCAN9_TX/MSC0_SDI2</t>
+          <t>PTC20/ADC3_SE2/FTU1_CH7/FLEXCAN9_TX/MSC0_SDI2</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2630,7 +2630,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ADC3_SE6/PTC21/FTU3_CH0/FLEXCAN9_RX/MSC0_SDI3</t>
+          <t>PTC21/ADC3_SE6/FTU3_CH0/FLEXCAN9_RX/MSC0_SDI3</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ADC3_SE10/PTC22/FTU3_CH1/FCUART17_RTS/MSC0_SDI1</t>
+          <t>PTC22/ADC3_SE10/FTU3_CH1/FCUART17_RTS/MSC0_SDI1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ADC2_SE0/PTC23/FTU6_CH6/FCUART2_RTS/FCUART12_TX/MSC0_SDI0</t>
+          <t>PTC23/ADC2_SE0/FTU6_CH6/FCUART2_RTS/FCUART12_TX/MSC0_SDI0</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2711,7 +2711,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ADC2_SE2/PTC24/FTU3_CH2/FLEXCAN6_RX/FCUART2_CTS</t>
+          <t>PTC24/ADC2_SE2/FTU3_CH2/FLEXCAN6_RX/FCUART2_CTS</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2738,7 +2738,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DISABLED/PTC25/FTU3_CH3/FCUART5_RTS/FCSPI5_PCS0/FLEXCAN2_TX</t>
+          <t>PTC25/DISABLED/FTU3_CH3/FCUART5_RTS/FCSPI5_PCS0/FLEXCAN2_TX</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2765,7 +2765,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DISABLED/PTC26/FTU9_CH7/FLEXCAN2_TX</t>
+          <t>PTC26/DISABLED/FTU9_CH7/FLEXCAN2_TX</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2787,7 +2787,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ADC2_SE7/PTC27/FTU10_CH5/FCSPI2_PCS1/FCUART5_RX</t>
+          <t>PTC27/ADC2_SE7/FTU10_CH5/FCSPI2_PCS1/FCUART5_RX</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2809,7 +2809,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ADC3_SE23/PTC28/FTU7_CH2/FLEXCAN3_TX/SDDF0_CLK0</t>
+          <t>PTC28/ADC3_SE23/FTU7_CH2/FLEXCAN3_TX/SDDF0_CLK0</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2836,7 +2836,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ADC2_SE10/PTC29/FTU7_CH5/FLEXCAN3_RX/SDDF0_CLK1</t>
+          <t>PTC29/ADC2_SE10/FTU7_CH5/FLEXCAN3_RX/SDDF0_CLK1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2863,7 +2863,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ADC2_SE12/PTC30/FTU7_CH7/FTU5_QD_PHA/FCSPI4_SOUT</t>
+          <t>PTC30/ADC2_SE12/FTU7_CH7/FTU5_QD_PHA/FCSPI4_SOUT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ADC2_SE14/PTC31/FTU5_CH1/FTU5_QD_PHB/TRGSEL_OUT3/SDDF0_CH1/FCSPI7_SCK</t>
+          <t>PTC31/ADC2_SE14/FTU5_CH1/FTU5_QD_PHB/TRGSEL_OUT3/SDDF0_CH1/FCSPI7_SCK</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2917,7 +2917,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ADC0_SE13/PTD0/FTU4_CH2/FCUART17_TX/TRGSEL_OUT1</t>
+          <t>PTD0/ADC0_SE13/FTU4_CH2/FCUART17_TX/TRGSEL_OUT1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2944,7 +2944,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ADC0_SE6/PTD1/FCUART6_TX/FTU2_CH4/TRGSEL_OUT2</t>
+          <t>PTD1/ADC0_SE6/FCUART6_TX/FTU2_CH4/TRGSEL_OUT2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2971,7 +2971,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DISABLED/PTD2/FTU2_CH0/FCSPI1_SCK</t>
+          <t>PTD2/DISABLED/FTU2_CH0/FCSPI1_SCK</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2998,7 +2998,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DISABLED/PTD3/FTU3_CH7/FCSPI1_SIN</t>
+          <t>PTD3/DISABLED/FTU3_CH7/FCSPI1_SIN</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3025,7 +3025,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DISABLED/PTD4/FTU3_CH6/FCSPI1_SOUT/FTU_FLT16</t>
+          <t>PTD4/DISABLED/FTU3_CH6/FCSPI1_SOUT/FTU_FLT16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3052,7 +3052,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DISABLED/PTD5/FTU6_CH4/FCUART2_CTS/TRACE_D2/ENET_TXD3/OSPI_A_IO5/FCSPI3_SIN</t>
+          <t>PTD5/DISABLED/FTU6_CH4/FCUART2_CTS/TRACE_D2/ENET_TXD3/OSPI_A_IO5/FCSPI3_SIN</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3079,7 +3079,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DISABLED/PTD6/FCUART2_RX/FLEXCAN3_RX/TRACE_D1/ENET_TXD2/OSPI_A_IO4/FCSPI3_SCK</t>
+          <t>PTD6/DISABLED/FCUART2_RX/FLEXCAN3_RX/TRACE_D1/ENET_TXD2/OSPI_A_IO4/FCSPI3_SCK</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DISABLED/PTD7/FCUART2_TX/FLEXCAN3_TX/TRACE_D0/ENET_TXD1</t>
+          <t>PTD7/DISABLED/FCUART2_TX/FLEXCAN3_TX/TRACE_D0/ENET_TXD1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3133,7 +3133,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DISABLED/PTD8/FTU7_CH0/FCSPI2_PCS2/FTU1_CH6/ENET_RX_DV_CTL/FCUART4_RX</t>
+          <t>PTD8/DISABLED/FTU7_CH0/FCSPI2_PCS2/FTU1_CH6/ENET_RX_DV_CTL/FCUART4_RX</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3160,7 +3160,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DISABLED/PTD9/FTU8_CH7/FCSPI2_PCS1/TRACE_D7/ENET_RXD2/OSPI_A_SCK/FCUART4_TX</t>
+          <t>PTD9/DISABLED/FTU8_CH7/FCSPI2_PCS1/TRACE_D7/ENET_RXD2/OSPI_A_SCK/FCUART4_TX</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3187,7 +3187,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DISABLED/PTD10/FTU6_CH7/FTU2_QD_PHB/ENET_RX_CLK</t>
+          <t>PTD10/DISABLED/FTU6_CH7/FTU2_QD_PHB/ENET_RX_CLK</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3214,7 +3214,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DISABLED/PTD11/FTU6_CH6/FTU2_QD_PHA/TRACE_D4/ENET_TX_CLK/OSPI_A_IO7</t>
+          <t>PTD11/DISABLED/FTU6_CH6/FTU2_QD_PHA/TRACE_D4/ENET_TX_CLK/OSPI_A_IO7</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3241,7 +3241,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>DISABLED/PTD12/FTU6_CH5/FCUART2_RTS/TRACE_D3/ENET_TX_EN_CTL/OSPI_A_IO6/FCSPI3_SOUT</t>
+          <t>PTD12/DISABLED/FTU6_CH5/FCUART2_RTS/TRACE_D3/ENET_TX_EN_CTL/OSPI_A_IO6/FCSPI3_SOUT</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3268,7 +3268,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ADC0_SE27/PTD15/FTU5_CH0/FLEXCAN2_RX/TRACE_D7/ENET_PPS2/FCUART2_RTS</t>
+          <t>PTD15/ADC0_SE27/FTU5_CH0/FLEXCAN2_RX/TRACE_D7/ENET_PPS2/FCUART2_RTS</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3295,7 +3295,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ADC0_SE26/PTD16/FTU5_CH1/FLEXCAN2_TX/TRACE_D6/FCSPI1_PCS3</t>
+          <t>PTD16/ADC0_SE26/FTU5_CH1/FLEXCAN2_TX/TRACE_D6/FCSPI1_PCS3</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3322,7 +3322,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ADC0_SE24/PTD17/FTU5_CH3/FCUART2_TX/TRACE_D4/FCSPI1_PCS1/FTU5_QD_PHA</t>
+          <t>PTD17/ADC0_SE24/FTU5_CH3/FCUART2_TX/TRACE_D4/FCSPI1_PCS1/FTU5_QD_PHA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3349,7 +3349,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ADC2_SE16/PTD18/FTU5_CH3/FCIIC1_SDA/SDDF0_CH3/FCSPI7_PCS0</t>
+          <t>PTD18/ADC2_SE16/FTU5_CH3/FCIIC1_SDA/SDDF0_CH3/FCSPI7_PCS0</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3376,7 +3376,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ADC2_SE17/PTD19/FTU5_CH4/FCIIC1_SCL/SDDF0_CLK2</t>
+          <t>PTD19/ADC2_SE17/FTU5_CH4/FCIIC1_SCL/SDDF0_CLK2</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3403,7 +3403,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ADC2_SE30/PTD20/FTU3_CH4/FCUART5_RX/FCSPI1_PCS1</t>
+          <t>PTD20/ADC2_SE30/FTU3_CH4/FCUART5_RX/FCSPI1_PCS1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ISP_EN_B/PTD21/FTU3_CH5/FCUART5_TX/FTU9_CH7</t>
+          <t>PTD21/ISP_EN_B/FTU3_CH5/FCUART5_TX/FTU9_CH7</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3457,7 +3457,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DISABLED/PTD22/FTU9_CH4/FCSPI5_SCK</t>
+          <t>PTD22/DISABLED/FTU9_CH4/FCSPI5_SCK</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3479,7 +3479,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ADC2_SE31/PTD23/FTU2_CH1/FCSPI1_PCS0</t>
+          <t>PTD23/ADC2_SE31/FTU2_CH1/FCSPI1_PCS0</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>DISABLED/PTD24/FTU2_CH4/MSC1_SOP/FCUART16_RX</t>
+          <t>PTD24/DISABLED/FTU2_CH4/MSC1_SOP/FCUART16_RX</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3533,7 +3533,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>DISABLED/PTD25/FTU2_CH6/FCUART12_TX/FCUART4_RTS/FLEXCAN7_TX</t>
+          <t>PTD25/DISABLED/FTU2_CH6/FCUART12_TX/FCUART4_RTS/FLEXCAN7_TX</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3560,7 +3560,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DISABLED/PTD26/FTU4_CH0/FLEXCAN0_TX/FCUART4_CTS</t>
+          <t>PTD26/DISABLED/FTU4_CH0/FLEXCAN0_TX/FCUART4_CTS</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>DISABLED/PTD27/FTU4_CH1/FLEXCAN0_RX/MSC1_EN0</t>
+          <t>PTD27/DISABLED/FTU4_CH1/FLEXCAN0_RX/MSC1_EN0</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3614,7 +3614,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DISABLED/PTD28/FTU4_CH3/FLEXCAN4_RX/FCUART11_TX</t>
+          <t>PTD28/DISABLED/FTU4_CH3/FLEXCAN4_RX/FCUART11_TX</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3641,7 +3641,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DISABLED/PTD29/FTU4_CH5/FCUART15_TX/SENT1_RXD1/FTU1_QD_PHB/MSC1_EN1</t>
+          <t>PTD29/DISABLED/FTU4_CH5/FCUART15_TX/SENT1_RXD1/FTU1_QD_PHB/MSC1_EN1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3668,7 +3668,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>DISABLED/PTD30/FTU4_CH7/FLEXCAN5_TX/SENT1_RXD3/FTU2_QD_PHB/MSC1_SDI1</t>
+          <t>PTD30/DISABLED/FTU4_CH7/FLEXCAN5_TX/SENT1_RXD3/FTU2_QD_PHB/MSC1_SDI1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3695,7 +3695,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ADC1_SE31/PTD31/FTU6_CH0/MSC1_SDI3/FTU1_QD_PHA</t>
+          <t>PTD31/ADC1_SE31/FTU6_CH0/MSC1_SDI3/FTU1_QD_PHA</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3722,7 +3722,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CMP1_IN4/PTE0/FCUART0_CTS/FTU_TCK1/FCIIC1_SDA/FCSPI0_SCK/FTU_FLT19</t>
+          <t>PTE0/CMP1_IN4/FCUART0_CTS/FTU_TCK1/FCIIC1_SDA/FCSPI0_SCK/FTU_FLT19</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CMP1_IN5/PTE1/FCUART0_RTS/FCIIC1_SCL/FCSPI0_SIN/FTU_FLT18</t>
+          <t>PTE1/CMP1_IN5/FCUART0_RTS/FCIIC1_SCL/FCSPI0_SIN/FTU_FLT18</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3776,7 +3776,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ADC1_SE24/PTE2/FTU6_CH6/FLEXCAN1_RX/FCUART1_CTS</t>
+          <t>PTE2/ADC1_SE24/FTU6_CH6/FLEXCAN1_RX/FCUART1_CTS</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3803,7 +3803,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>OSC32K_EXTAL/PTE3/FTU0_CH2/FTU_FLT1/FTU_TCK0</t>
+          <t>PTE3/OSC32K_EXTAL/FTU0_CH2/FTU_FLT1/FTU_TCK0</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3830,7 +3830,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CMP0_IN0/PTE4/FTU2_QD_PHB/FTU10_CH7/FCUART7_TX</t>
+          <t>PTE4/CMP0_IN0/FTU2_QD_PHB/FTU10_CH7/FCUART7_TX</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ADC0_SE12/PTE5/FTU_TCK2/FTU4_CH3/FCSPI2_PCS1/FCUART17_RX</t>
+          <t>PTE5/ADC0_SE12/FTU_TCK2/FTU4_CH3/FCSPI2_PCS1/FCUART17_RX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3884,7 +3884,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ADC1_SE25/PTE6/FTU6_CH5/FLEXCAN1_TX/FCUART1_RTS</t>
+          <t>PTE6/ADC1_SE25/FTU6_CH5/FLEXCAN1_TX/FCUART1_RTS</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3911,7 +3911,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ADC2_SE15/PTE7/FTU5_CH2/FTU_FLT14/SDDF0_CH2/FCSPI7_SOUT</t>
+          <t>PTE7/ADC2_SE15/FTU5_CH2/FTU_FLT14/SDDF0_CH2/FCSPI7_SOUT</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3938,7 +3938,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>DISABLED/PTE8/FTU6_CH1/FCUART9_RX/ENET_MDC/FCSPI3_SCK</t>
+          <t>PTE8/DISABLED/FTU6_CH1/FCUART9_RX/ENET_MDC/FCSPI3_SCK</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3965,7 +3965,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ADC0_SE28/PTE9/FTU0_CH7/TRACE_CLKOUT/ENET_PPS3/FCUART2_CTS</t>
+          <t>PTE9/ADC0_SE28/FTU0_CH7/TRACE_CLKOUT/ENET_PPS3/FCUART2_CTS</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3992,7 +3992,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ADC0_SE9/PTE10/SCG_CLKOUT/FTU6_CH0/FCSPI2_SIN/TRGSEL_OUT4</t>
+          <t>PTE10/ADC0_SE9/SCG_CLKOUT/FTU6_CH0/FCSPI2_SIN/TRGSEL_OUT4</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4019,7 +4019,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ADC0_SE8/PTE11/FTU2_CH1/FCSPI2_PCS0/TRGSEL_OUT5</t>
+          <t>PTE11/ADC0_SE8/FTU2_CH1/FCSPI2_PCS0/TRGSEL_OUT5</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -4046,7 +4046,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ADC0_SE17/PTE12/FTU5_CH6/FTU_FLT2/TRACE_D3/FCSPI1_SOUT</t>
+          <t>PTE12/ADC0_SE17/FTU5_CH6/FTU_FLT2/TRACE_D3/FCSPI1_SOUT</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ADC0_SE10/PTE13/FTU2_CH0/FCSPI2_SCK</t>
+          <t>PTE13/ADC0_SE10/FTU2_CH0/FCSPI2_SCK</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -4100,7 +4100,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>OSC32K_XTAL/PTE14/FTU0_CH3/FTU_FLT0</t>
+          <t>PTE14/OSC32K_XTAL/FTU0_CH3/FTU_FLT0</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ADC0_SE5/PTE15/FCUART1_CTS/FLEXCAN5_RX/FTU2_CH6/TRGSEL_OUT6</t>
+          <t>PTE15/ADC0_SE5/FCUART1_CTS/FLEXCAN5_RX/FTU2_CH6/TRGSEL_OUT6</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -4154,7 +4154,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ADC1_SE2/PTE16/FCUART1_RTS/FLEXCAN5_TX/FTU2_CH7/TRGSEL_OUT7</t>
+          <t>PTE16/ADC1_SE2/FCUART1_RTS/FLEXCAN5_TX/FTU2_CH7/TRGSEL_OUT7</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -4181,7 +4181,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>DISABLED/PTE17/FTU6_CH1/FCSMU_PIN1</t>
+          <t>PTE17/DISABLED/FTU6_CH1/FCSMU_PIN1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -4208,7 +4208,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ADC1_SE29/PTE18/FTU6_CH3/FTU5_QD_PHA/FCUART10_RX/FLEXCAN3_TX</t>
+          <t>PTE18/ADC1_SE29/FTU6_CH3/FTU5_QD_PHA/FCUART10_RX/FLEXCAN3_TX</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -4235,7 +4235,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ADC1_SE23/PTE19/SCG_CLKOUT/FCIIC0_SCL/SENT0_RXD2/CMP0_OUT</t>
+          <t>PTE19/ADC1_SE23/SCG_CLKOUT/FCIIC0_SCL/SENT0_RXD2/CMP0_OUT</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -4262,7 +4262,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ADC1_SE22/PTE20/FTU0_CH0/FCIIC0_SDA/SENT0_RXD3</t>
+          <t>PTE20/ADC1_SE22/FTU0_CH0/FCIIC0_SDA/SENT0_RXD3</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -4289,7 +4289,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ADC1_SE21/PTE21/FTU0_CH1/FLEXCAN0_TX/FCUART0_RTS</t>
+          <t>PTE21/ADC1_SE21/FTU0_CH1/FLEXCAN0_TX/FCUART0_RTS</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -4316,7 +4316,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ADC1_SE20/PTE22/FTU0_CH2/FLEXCAN0_RX/FCUART0_CTS</t>
+          <t>PTE22/ADC1_SE20/FTU0_CH2/FLEXCAN0_RX/FCUART0_CTS</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -4343,7 +4343,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>CMP1_IN6/PTE23/FTU0_CH4/FLEXCAN1_RX/CMP2_OUT/FCSPI0_PCS2</t>
+          <t>PTE23/CMP1_IN6/FTU0_CH4/FLEXCAN1_RX/CMP2_OUT/FCSPI0_PCS2</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4370,7 +4370,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CMP1_IN7/PTE24/FTU0_CH5/FLEXCAN1_TX/FCSPI0_PCS1</t>
+          <t>PTE24/CMP1_IN7/FTU0_CH5/FLEXCAN1_TX/FCSPI0_PCS1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ADC1_SE19/PTE25/FTU0_CH6/AONTIMER0_CLK0/FCSPI0_PCS0/TRGSEL_OUT7</t>
+          <t>PTE25/ADC1_SE19/FTU0_CH6/AONTIMER0_CLK0/FCSPI0_PCS0/TRGSEL_OUT7</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4424,7 +4424,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ADC1_SE17/PTE26/FTU3_CH2/AONTIMER0_CLK2/SENT0_RXD0</t>
+          <t>PTE26/ADC1_SE17/FTU3_CH2/AONTIMER0_CLK2/SENT0_RXD0</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4451,7 +4451,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ADC1_SE16/PTE27/FTU3_CH5/SENT0_RXD1</t>
+          <t>PTE27/ADC1_SE16/FTU3_CH5/SENT0_RXD1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">

</xml_diff>

<commit_message>
feat(pinout): GPIO multi-function pins LEFT, group PWR, drop empty-Ball rows
</commit_message>
<xml_diff>
--- a/pinout/fc7300-320-pin-a1.xlsx
+++ b/pinout/fc7300-320-pin-a1.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -471,7 +471,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1334,12 +1334,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VREFH_0</t>
+          <t>VDDA_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>H8</t>
+          <t>N11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1349,24 +1349,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>84</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VREFL_0</t>
+          <t>VREFH_0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>J8</t>
+          <t>H8</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>V15_CFG</t>
+          <t>VREFH_1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>N12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1403,24 +1403,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>85</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>V15_BASE_DRIVER</t>
+          <t>VREFL_0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>J8</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1435,19 +1435,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>V11_0</t>
+          <t>VREFL_1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>N13</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1457,24 +1457,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>86</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>V15_0</t>
+          <t>V15_CFG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1489,19 +1489,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VDD_HV_A_1</t>
+          <t>V15_BASE_DRIVER</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1516,19 +1516,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>V25</t>
+          <t>V11_0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>L6</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1543,19 +1543,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VDD_HV_A_2</t>
+          <t>V11_1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>H12</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1565,24 +1565,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>74</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VDD_HV_B_1</t>
+          <t>V11_2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>T7</t>
+          <t>J13</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1592,24 +1592,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>112</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>VDD_HV_B_2</t>
+          <t>V11_3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>T9</t>
+          <t>H10</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1619,24 +1619,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LEFT</t>
+          <t>RIGHT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>153</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VDD_HV_A_3</t>
+          <t>V15_0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>L8</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V11_1</t>
+          <t>V15_2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>K13</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1705,19 +1705,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>111</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VDD_HV_A_4</t>
+          <t>V15_3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>L13</t>
+          <t>H11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1728,18 +1728,23 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>RIGHT</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>152</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VDDA_1</t>
+          <t>VDD_HV_A_1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>N11</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1749,24 +1754,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VREFH_1</t>
+          <t>VDD_HV_A_2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>N12</t>
+          <t>H12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1776,24 +1781,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VREFL_1</t>
+          <t>VDD_HV_A_3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>N13</t>
+          <t>L8</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1803,24 +1808,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>72</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VDD_HV_A_5</t>
+          <t>VDD_HV_A_4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>N10</t>
+          <t>L13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1831,23 +1836,18 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>RIGHT</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>92</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VDD_HV_A_6</t>
+          <t>VDD_HV_A_5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>N10</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1862,19 +1862,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>92</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>V15_2</t>
+          <t>VDD_HV_A_6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>K13</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1889,19 +1889,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>V11_2</t>
+          <t>V25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>J13</t>
+          <t>L6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1911,22 +1911,26 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VDD_HV_A_7</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>VDD_HV_B_1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>PWR</t>
@@ -1934,22 +1938,26 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>53</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VDD_HV_A_8</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
+          <t>VDD_HV_B_2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>PWR</t>
@@ -1957,112 +1965,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RIGHT</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>141</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>VDD_HV_A_9</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>RIGHT</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>151</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>V15_3</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>RIGHT</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>V11_3</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>RIGHT</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>153</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>VDD_HV_A_10</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>PWR</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>RIGHT</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>176</t>
+          <t>61</t>
         </is>
       </c>
     </row>
@@ -2105,12 +2013,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VSS_1</t>
+          <t>VSSA_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>M13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2121,23 +2029,18 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>LEFT</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>177</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VSS_2</t>
+          <t>VSS_1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A20</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2159,12 +2062,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VSS_3</t>
+          <t>VSS_2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>A20</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2186,12 +2089,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VSS_4</t>
+          <t>VSS_3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2213,12 +2116,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VSS_5</t>
+          <t>VSS_4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>B19</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2240,12 +2143,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>VSS_6</t>
+          <t>VSS_5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2267,12 +2170,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VSS_7</t>
+          <t>VSS_6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2294,12 +2197,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>VSS_8</t>
+          <t>VSS_7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2321,12 +2224,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>VSSA_1</t>
+          <t>VSS_8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2337,6 +2240,11 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>LEFT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>177</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3102,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -3221,7 +3129,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3248,7 +3156,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3275,7 +3183,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3302,7 +3210,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3329,7 +3237,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3356,7 +3264,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3383,7 +3291,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3410,7 +3318,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3437,7 +3345,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3464,7 +3372,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3394,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3513,7 +3421,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3540,7 +3448,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3567,7 +3475,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3594,7 +3502,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3621,7 +3529,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3648,7 +3556,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3675,7 +3583,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3702,7 +3610,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3729,7 +3637,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3756,7 +3664,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3783,7 +3691,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -3810,7 +3718,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3837,7 +3745,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3864,7 +3772,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3891,7 +3799,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3918,7 +3826,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3945,7 +3853,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3972,7 +3880,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4013,7 +3921,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -4040,7 +3948,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4067,7 +3975,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4094,7 +4002,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4121,7 +4029,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4148,7 +4056,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4175,7 +4083,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4202,7 +4110,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4229,7 +4137,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4256,7 +4164,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4283,7 +4191,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4310,7 +4218,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4337,7 +4245,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4364,7 +4272,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4391,7 +4299,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4418,7 +4326,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4445,7 +4353,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4472,7 +4380,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4499,7 +4407,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4526,7 +4434,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4553,7 +4461,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4580,7 +4488,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4607,7 +4515,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4634,7 +4542,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4661,7 +4569,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4688,7 +4596,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -4715,7 +4623,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4645,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4667,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -4786,7 +4694,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4813,7 +4721,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -4840,7 +4748,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4881,7 +4789,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -4908,7 +4816,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4935,7 +4843,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4962,7 +4870,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4989,7 +4897,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5016,7 +4924,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5043,7 +4951,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5070,7 +4978,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5097,7 +5005,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5124,7 +5032,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5151,7 +5059,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5178,7 +5086,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5205,7 +5113,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5232,7 +5140,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5259,7 +5167,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5286,7 +5194,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5313,7 +5221,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5340,7 +5248,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5367,7 +5275,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5394,7 +5302,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5421,7 +5329,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -5443,7 +5351,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5470,7 +5378,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5497,7 +5405,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5524,7 +5432,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5551,7 +5459,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5578,7 +5486,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5605,7 +5513,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5632,7 +5540,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5659,7 +5567,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5700,7 +5608,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -5727,7 +5635,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5754,7 +5662,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5781,7 +5689,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5808,7 +5716,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5835,7 +5743,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5862,7 +5770,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5889,7 +5797,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5916,7 +5824,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5943,7 +5851,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5970,7 +5878,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5997,7 +5905,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6024,7 +5932,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6051,7 +5959,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6078,7 +5986,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6105,7 +6013,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6132,7 +6040,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6159,7 +6067,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -6186,7 +6094,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6213,7 +6121,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6240,7 +6148,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6267,7 +6175,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6294,7 +6202,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6321,7 +6229,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6348,7 +6256,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -6375,7 +6283,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6402,7 +6310,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6429,7 +6337,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6470,7 +6378,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6400,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6422,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6444,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6558,7 +6466,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6580,7 +6488,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6510,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6532,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6646,7 +6554,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6668,7 +6576,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6690,7 +6598,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6712,7 +6620,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6642,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6664,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6778,7 +6686,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6708,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6822,7 +6730,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6752,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6774,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6796,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6910,7 +6818,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6932,7 +6840,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6954,7 +6862,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6884,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6906,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7034,7 +6942,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7056,7 +6964,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7078,7 +6986,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7008,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7030,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7144,7 +7052,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7074,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7096,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7118,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7140,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7162,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7184,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7206,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7320,7 +7228,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7342,7 +7250,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7364,7 +7272,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7386,7 +7294,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7316,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7430,7 +7338,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7452,7 +7360,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7382,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7404,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7518,7 +7426,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7540,7 +7448,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7576,7 +7484,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7506,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7620,7 +7528,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7642,7 +7550,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7572,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7686,7 +7594,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7708,7 +7616,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7730,7 +7638,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7660,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7774,7 +7682,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7704,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7818,7 +7726,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7748,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7862,7 +7770,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7792,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7906,7 +7814,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7928,7 +7836,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7950,7 +7858,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7880,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7902,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8016,7 +7924,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8038,7 +7946,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8060,7 +7968,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8082,7 +7990,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8118,7 +8026,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8140,7 +8048,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8162,7 +8070,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8184,7 +8092,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8206,7 +8114,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8228,7 +8136,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8250,7 +8158,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8180,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8202,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8316,7 +8224,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8338,7 +8246,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8360,7 +8268,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8382,7 +8290,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8312,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8426,7 +8334,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8448,7 +8356,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8378,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8492,7 +8400,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8514,7 +8422,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8444,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8558,7 +8466,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8580,7 +8488,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8602,7 +8510,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>
@@ -8624,7 +8532,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Right</t>
+          <t>LEFT</t>
         </is>
       </c>
     </row>

</xml_diff>